<commit_message>
modifico tablas testeosv2 y exploratoria
</commit_message>
<xml_diff>
--- a/tests/Prueba_exploratoria.xlsx
+++ b/tests/Prueba_exploratoria.xlsx
@@ -4,13 +4,15 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="9240" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="5280" yWindow="0" windowWidth="22260" windowHeight="12645"/>
   </bookViews>
   <sheets>
-    <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
+    <sheet name="Exploratorio Sprint 2 " sheetId="2" r:id="rId1"/>
+    <sheet name="Exploratorio Sprint 1" sheetId="1" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$E$3:$F$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Exploratorio Sprint 1'!$E$3:$F$35</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Exploratorio Sprint 2 '!$F$3:$G$39</definedName>
   </definedNames>
   <calcPr calcId="162913"/>
   <extLst>
@@ -22,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="346" uniqueCount="74">
   <si>
     <t>#</t>
   </si>
@@ -132,6 +134,9 @@
     <t>EL HEADER INCLUYE A IZQUIERDA LOGO Y LEMA CLICKEABLES</t>
   </si>
   <si>
+    <t>pendiente, se ve mal el texto de la card</t>
+  </si>
+  <si>
     <t>no hay pagina, se usó Modal</t>
   </si>
   <si>
@@ -153,19 +158,94 @@
     <t>x</t>
   </si>
   <si>
+    <t>No se pudo probar por falla de logueo</t>
+  </si>
+  <si>
     <t>Boton dice "ver más"</t>
   </si>
   <si>
     <t>Se usa Modal. De fondo el Header y el Buscador</t>
   </si>
   <si>
+    <t>pendiente ver botones en categoria</t>
+  </si>
+  <si>
     <t>no hay pagina, se usó Modal. De fondo se ve.</t>
   </si>
   <si>
-    <t>Por ahora hay una sóla Pagina</t>
-  </si>
-  <si>
-    <t>pendiente, ver texto de card y header</t>
+    <t>comentarios spring1</t>
+  </si>
+  <si>
+    <t>S1</t>
+  </si>
+  <si>
+    <t>PAGINA PRODUCTO</t>
+  </si>
+  <si>
+    <t>S2</t>
+  </si>
+  <si>
+    <t>AL SELECCIONAR UN VEHICULO E INGRESAR A LA PAGINA SE OBTIENE UNA URL AMIGABLE</t>
+  </si>
+  <si>
+    <t>DESDE LA PAGINA DE PRODUCTO PUEDO SALIR ( FLECHA ATRÁS) HACIA LA HOME.</t>
+  </si>
+  <si>
+    <t>CONTIENE LOS SIGUIENTES BLOQUES: HEADER, UBICACIÓN, IMÁGENES, DESCRIPCION, CARACTERISTICAS, POLITICAS, RESERVAS</t>
+  </si>
+  <si>
+    <t>EL BLOQUE HEADER CONTIENE LA CATEGORIA DEL PRODUCTO, EL TITULO Y UNA FLECHA BACK</t>
+  </si>
+  <si>
+    <t>EL BLOQUE UBICACION CONTIENE LA UBICACIÓN DEL PRODUCTO</t>
+  </si>
+  <si>
+    <t>EN FORMATO DESKTOP EL BLOQUE IMÁGENES CONTIENE  5 IMÁGENES UNA GRANDE Y OTRAS 4 MAS CHICAS EN GRILLA DE 2 X2 , CON BORDES REDONDEADOS Y UN BOTON QUE DICE "VER MAS" PARA ACCEDER A MAS FOTOS.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">EN FORMATO TABLET EL BLOQUE IMÁGENES CONTIENE  1 IMAGEN  QUE CUBRE EL 100% DEL ANCHO Y LA IMAGEN CAMBIAS CADA 3 SEGUNDOS. DEBAJO UN INDICADOR CON EL NUMERO DE FOTO ACTUAL Y EL TOTAL DE IMAGENES. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">EN FORMATO PHONE EL BLOQUE IMÁGENES CONTIENE  1 IMAGEN  QUE CUBRE EL 100% DEL ANCHO Y LA IMAGEN CAMBIAS CADA 3 SEGUNDOS. DEBAJO UN INDICADOR CON EL NUMERO DE FOTO ACTUAL Y EL TOTAL DE IMAGENES. </t>
+  </si>
+  <si>
+    <t xml:space="preserve">EN FORMATO DESKTOP, EL BLOQUE CARACTERISTICAS CONTIENE EL TITULO Y UNA GRILLA DE 4 COLUMNAS CON ATRIBUTOS ASOCIADOS A SU ICONO CORRESPONDIENTE.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">EN FORMATO TABLET, EL BLOQUE CARACTERISTICAS CONTIENE EL TITULO Y UNA GRILLA DE 2 COLUMNAS CON ATRIBUTOS ASOCIADOS A SU ICONO CORRESPONDIENTE.  </t>
+  </si>
+  <si>
+    <t xml:space="preserve">EN FORMATO PHONE, EL BLOQUE CARACTERISTICAS CONTIENE EL TITULO Y UNA GRILLA DE 1 COLUMNA CON ATRIBUTOS ASOCIADOS A SU ICONO CORRESPONDIENTE.  </t>
+  </si>
+  <si>
+    <t>EL BLOQUE DESCRIPCION CONTIENE EL TITULO Y UN TEXTO DE DESCRIPCION. ES RESPONSIVE A TABLET Y PHONE</t>
+  </si>
+  <si>
+    <t>EN FORMATO DESKTOP, EL BLOQUE POLITICAS  CONTIENE EL TITULO Y UNA GRILLA DE 3 COLUMNAS Y EN CADA UNA UN TITULO Y UNA DESCRPICON.</t>
+  </si>
+  <si>
+    <t>EN FORMATO TABLET, EL BLOQUE POLITICAS  CONTIENE EL TITULO Y UNA GRILLA DE 2 COLUMNAS Y EN CADA UNA UN TITULO Y UNA DESCRPICON.</t>
+  </si>
+  <si>
+    <t>EN FORMATO PHONE, EL BLOQUE POLITICAS  CONTIENE EL TITULO Y UNA GRILLA DE 1 COLUMNA Y EN CADA UNA UN TITULO Y UNA DESCRPICON.</t>
+  </si>
+  <si>
+    <t>EN FORMATO DESKTOP, EL BLOQUE RESERVAS CONTIENE UN CALENDARIO ALINEADO A IZQUIERDA QUE MUESTRE 2 MESES E INDICA TANTO LAS FECHAS DISPONIBLES COMO LAS NO DISPONIBLES. AL LADO UN BOTON DE INICIAR RESERVA.</t>
+  </si>
+  <si>
+    <t>EN FORMATO TABLET, EL BLOQUE RESERVAS CONTIENE UN CALENDARIO ALINEADO A IZQUIERDA QUE MUESTRE 2 MESES E INDCA TANTO LAS FECHAS DISPONIBLES COMO LAS NO DISPONIBLES. DEBAJO UN BOTON DE INICIAR RESERVA.</t>
+  </si>
+  <si>
+    <t>EN FORMATO TABLET, EL BLOQUE RESERVAS CONTIENE UN CALENDARIO ALINEADO A IZQUIERDA QUE MUESTRE 1 MES E INDCA TANTO LAS FECHAS DISPONIBLES COMO LAS NO DISPONIBLES. DEBAJO UN BOTON DE INICIAR RESERVA.</t>
+  </si>
+  <si>
+    <t>AL INICIAR LA PAGINA ME MUESTRA UN GRUPO RANDOM DE VEHICULOS, REINICIANDO SE MODIFICAN</t>
+  </si>
+  <si>
+    <t>SELECCIONANDO UNA CIUDAD Y PRESIONANDO BUSCAR NO RENDERIZA LSO PRODUCTOS DIPONIBLES EN ESA CIUDAD</t>
+  </si>
+  <si>
+    <t>CREADO</t>
   </si>
 </sst>
 </file>
@@ -195,7 +275,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="18">
     <border>
       <left/>
       <right/>
@@ -334,11 +414,85 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -384,6 +538,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -401,6 +558,38 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="17" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -682,6 +871,1142 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B1:I59"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="3.5703125" customWidth="1"/>
+    <col min="2" max="2" width="7.140625" style="1" customWidth="1"/>
+    <col min="3" max="3" width="19.28515625" customWidth="1"/>
+    <col min="4" max="4" width="54.42578125" customWidth="1"/>
+    <col min="5" max="5" width="10.28515625" customWidth="1"/>
+    <col min="6" max="7" width="9.140625" style="1"/>
+    <col min="8" max="8" width="45.5703125" customWidth="1"/>
+    <col min="9" max="9" width="22.85546875" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
+    <row r="2" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B2" s="20" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="22" t="s">
+        <v>5</v>
+      </c>
+      <c r="D2" s="22" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="24"/>
+      <c r="F2" s="31" t="s">
+        <v>1</v>
+      </c>
+      <c r="G2" s="32"/>
+      <c r="H2" s="33"/>
+    </row>
+    <row r="3" spans="2:9" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B3" s="21"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
+      <c r="E3" s="17" t="s">
+        <v>73</v>
+      </c>
+      <c r="F3" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="G3" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="H3" s="28" t="s">
+        <v>39</v>
+      </c>
+      <c r="I3" s="26" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="4" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B4" s="3">
+        <v>1</v>
+      </c>
+      <c r="C4" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D4" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E4" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F4" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G4" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="5" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B5" s="3">
+        <v>2</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E5" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F5" s="13"/>
+      <c r="G5" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="6" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B6" s="3">
+        <v>33</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>6</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F6" s="13"/>
+      <c r="G6" s="13"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="25"/>
+    </row>
+    <row r="7" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B7" s="3">
+        <v>34</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="E7" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" s="13"/>
+      <c r="G7" s="13"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="25"/>
+    </row>
+    <row r="8" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B8" s="3">
+        <v>3</v>
+      </c>
+      <c r="C8" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D8" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G8" s="13"/>
+      <c r="H8" s="2"/>
+    </row>
+    <row r="9" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B9" s="3">
+        <v>4</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E9" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F9" s="13"/>
+      <c r="G9" s="13"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="10" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B10" s="3">
+        <v>5</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>10</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E10" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F10" s="13"/>
+      <c r="G10" s="13"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="11" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B11" s="3">
+        <v>35</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E11" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F11" s="13"/>
+      <c r="G11" s="13"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="25"/>
+    </row>
+    <row r="12" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B12" s="3">
+        <v>6</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="E12" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F12" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G12" s="13"/>
+      <c r="H12" s="2"/>
+    </row>
+    <row r="13" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B13" s="3">
+        <v>7</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="E13" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" s="13"/>
+      <c r="G13" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="14" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B14" s="3">
+        <v>8</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E14" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F14" s="13"/>
+      <c r="G14" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="15" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B15" s="4">
+        <v>9</v>
+      </c>
+      <c r="C15" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="8" t="s">
+        <v>40</v>
+      </c>
+      <c r="E15" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F15" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G15" s="13"/>
+      <c r="H15" s="2"/>
+    </row>
+    <row r="16" spans="2:9" ht="32.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="4">
+        <v>10</v>
+      </c>
+      <c r="C16" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D16" s="8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F16" s="13"/>
+      <c r="G16" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="17" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B17" s="3">
+        <v>11</v>
+      </c>
+      <c r="C17" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="E17" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F17" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G17" s="13"/>
+      <c r="H17" s="2"/>
+    </row>
+    <row r="18" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B18" s="4">
+        <v>12</v>
+      </c>
+      <c r="C18" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D18" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E18" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F18" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G18" s="13"/>
+      <c r="H18" s="2"/>
+    </row>
+    <row r="19" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B19" s="4">
+        <v>13</v>
+      </c>
+      <c r="C19" s="34" t="s">
+        <v>9</v>
+      </c>
+      <c r="D19" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E19" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F19" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G19" s="13"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B20" s="4"/>
+      <c r="C20" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D20" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E20" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F20" s="13"/>
+      <c r="G20" s="13"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+    </row>
+    <row r="21" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B21" s="3">
+        <v>14</v>
+      </c>
+      <c r="C21" s="34" t="s">
+        <v>10</v>
+      </c>
+      <c r="D21" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G21" s="13"/>
+      <c r="H21" s="2"/>
+      <c r="I21" s="2" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="22" spans="2:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="B22" s="4">
+        <v>15</v>
+      </c>
+      <c r="C22" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D22" s="8" t="s">
+        <v>16</v>
+      </c>
+      <c r="E22" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F22" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G22" s="13"/>
+      <c r="H22" s="2"/>
+    </row>
+    <row r="23" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B23" s="3">
+        <v>16</v>
+      </c>
+      <c r="C23" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D23" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="E23" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F23" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G23" s="13"/>
+      <c r="H23" s="2"/>
+    </row>
+    <row r="24" spans="2:9" x14ac:dyDescent="0.25">
+      <c r="B24" s="4">
+        <v>17</v>
+      </c>
+      <c r="C24" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" s="8" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F24" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G24" s="13"/>
+      <c r="H24" s="2"/>
+    </row>
+    <row r="25" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B25" s="3">
+        <v>18</v>
+      </c>
+      <c r="C25" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D25" s="8" t="s">
+        <v>18</v>
+      </c>
+      <c r="E25" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F25" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G25" s="13"/>
+      <c r="H25" s="2"/>
+    </row>
+    <row r="26" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B26" s="4">
+        <v>19</v>
+      </c>
+      <c r="C26" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D26" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F26" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G26" s="13"/>
+      <c r="H26" s="2"/>
+    </row>
+    <row r="27" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="3">
+        <v>20</v>
+      </c>
+      <c r="C27" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D27" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="E27" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F27" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G27" s="13"/>
+      <c r="H27" s="2"/>
+    </row>
+    <row r="28" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B28" s="4">
+        <v>21</v>
+      </c>
+      <c r="C28" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D28" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="E28" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F28" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G28" s="13"/>
+      <c r="H28" s="2"/>
+    </row>
+    <row r="29" spans="2:9" ht="50.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B29" s="3">
+        <v>22</v>
+      </c>
+      <c r="C29" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D29" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="E29" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F29" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G29" s="13"/>
+      <c r="H29" s="2"/>
+    </row>
+    <row r="30" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B30" s="4">
+        <v>23</v>
+      </c>
+      <c r="C30" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D30" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="E30" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F30" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G30" s="13"/>
+      <c r="H30" s="2"/>
+    </row>
+    <row r="31" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B31" s="3">
+        <v>24</v>
+      </c>
+      <c r="C31" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D31" s="8" t="s">
+        <v>24</v>
+      </c>
+      <c r="E31" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F31" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G31" s="13"/>
+      <c r="H31" s="2"/>
+      <c r="I31" s="2" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="32" spans="2:9" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B32" s="4">
+        <v>25</v>
+      </c>
+      <c r="C32" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="D32" s="8" t="s">
+        <v>26</v>
+      </c>
+      <c r="E32" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G32" s="13"/>
+      <c r="H32" s="2"/>
+      <c r="I32" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="33" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B33" s="3">
+        <v>26</v>
+      </c>
+      <c r="C33" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="D33" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E33" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F33" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G33" s="13"/>
+      <c r="H33" s="2"/>
+      <c r="I33" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="34" spans="2:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="B34" s="4">
+        <v>27</v>
+      </c>
+      <c r="C34" s="34" t="s">
+        <v>28</v>
+      </c>
+      <c r="D34" s="8" t="s">
+        <v>29</v>
+      </c>
+      <c r="E34" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F34" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G34" s="13"/>
+      <c r="H34" s="2"/>
+      <c r="I34" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="35" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B35" s="3">
+        <v>28</v>
+      </c>
+      <c r="C35" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="D35" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="E35" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F35" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G35" s="13"/>
+      <c r="H35" s="2"/>
+      <c r="I35" s="2" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="36" spans="2:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="B36" s="4">
+        <v>29</v>
+      </c>
+      <c r="C36" s="34" t="s">
+        <v>25</v>
+      </c>
+      <c r="D36" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="E36" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F36" s="13"/>
+      <c r="G36" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="H36" s="2"/>
+      <c r="I36" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="37" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B37" s="3">
+        <v>30</v>
+      </c>
+      <c r="C37" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D37" s="8" t="s">
+        <v>32</v>
+      </c>
+      <c r="E37" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F37" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G37" s="13"/>
+      <c r="H37" s="2"/>
+      <c r="I37" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="38" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B38" s="4">
+        <v>31</v>
+      </c>
+      <c r="C38" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D38" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="E38" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F38" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="G38" s="13"/>
+      <c r="H38" s="2"/>
+      <c r="I38" s="2" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="39" spans="2:9" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B39" s="4">
+        <v>32</v>
+      </c>
+      <c r="C39" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D39" s="8" t="s">
+        <v>34</v>
+      </c>
+      <c r="E39" s="13" t="s">
+        <v>50</v>
+      </c>
+      <c r="F39" s="13"/>
+      <c r="G39" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="H39" s="2"/>
+      <c r="I39" s="27" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="40" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B40" s="4">
+        <v>36</v>
+      </c>
+      <c r="C40" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D40" s="8" t="s">
+        <v>53</v>
+      </c>
+      <c r="E40" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F40" s="13"/>
+      <c r="G40" s="13"/>
+      <c r="H40" s="2"/>
+    </row>
+    <row r="41" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B41" s="4">
+        <v>37</v>
+      </c>
+      <c r="C41" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D41" s="8" t="s">
+        <v>54</v>
+      </c>
+      <c r="E41" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F41" s="13"/>
+      <c r="G41" s="13"/>
+      <c r="H41" s="2"/>
+    </row>
+    <row r="42" spans="2:9" ht="45" x14ac:dyDescent="0.25">
+      <c r="B42" s="4">
+        <v>38</v>
+      </c>
+      <c r="C42" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D42" s="8" t="s">
+        <v>55</v>
+      </c>
+      <c r="E42" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F42" s="13"/>
+      <c r="G42" s="13"/>
+      <c r="H42" s="2"/>
+    </row>
+    <row r="43" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B43" s="4">
+        <v>39</v>
+      </c>
+      <c r="C43" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D43" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="E43" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F43" s="13"/>
+      <c r="G43" s="13"/>
+      <c r="H43" s="2"/>
+    </row>
+    <row r="44" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B44" s="4">
+        <v>40</v>
+      </c>
+      <c r="C44" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D44" s="8" t="s">
+        <v>57</v>
+      </c>
+      <c r="E44" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F44" s="13"/>
+      <c r="G44" s="13"/>
+      <c r="H44" s="2"/>
+    </row>
+    <row r="45" spans="2:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="B45" s="4">
+        <v>41</v>
+      </c>
+      <c r="C45" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D45" s="8" t="s">
+        <v>58</v>
+      </c>
+      <c r="E45" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F45" s="13"/>
+      <c r="G45" s="13"/>
+      <c r="H45" s="2"/>
+    </row>
+    <row r="46" spans="2:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="B46" s="4">
+        <v>42</v>
+      </c>
+      <c r="C46" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D46" s="8" t="s">
+        <v>59</v>
+      </c>
+      <c r="E46" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F46" s="13"/>
+      <c r="G46" s="13"/>
+      <c r="H46" s="2"/>
+    </row>
+    <row r="47" spans="2:9" ht="60" x14ac:dyDescent="0.25">
+      <c r="B47" s="4">
+        <v>43</v>
+      </c>
+      <c r="C47" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D47" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="E47" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F47" s="13"/>
+      <c r="G47" s="13"/>
+      <c r="H47" s="2"/>
+    </row>
+    <row r="48" spans="2:9" ht="30" x14ac:dyDescent="0.25">
+      <c r="B48" s="4">
+        <v>44</v>
+      </c>
+      <c r="C48" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D48" s="8" t="s">
+        <v>64</v>
+      </c>
+      <c r="E48" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F48" s="13"/>
+      <c r="G48" s="13"/>
+      <c r="H48" s="2"/>
+    </row>
+    <row r="49" spans="2:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="B49" s="4">
+        <v>45</v>
+      </c>
+      <c r="C49" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D49" s="8" t="s">
+        <v>61</v>
+      </c>
+      <c r="E49" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F49" s="13"/>
+      <c r="G49" s="13"/>
+      <c r="H49" s="2"/>
+    </row>
+    <row r="50" spans="2:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="B50" s="4">
+        <v>46</v>
+      </c>
+      <c r="C50" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D50" s="8" t="s">
+        <v>62</v>
+      </c>
+      <c r="E50" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F50" s="13"/>
+      <c r="G50" s="13"/>
+      <c r="H50" s="2"/>
+    </row>
+    <row r="51" spans="2:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="B51" s="4">
+        <v>47</v>
+      </c>
+      <c r="C51" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D51" s="8" t="s">
+        <v>63</v>
+      </c>
+      <c r="E51" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F51" s="13"/>
+      <c r="G51" s="13"/>
+      <c r="H51" s="2"/>
+    </row>
+    <row r="52" spans="2:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="B52" s="4">
+        <v>48</v>
+      </c>
+      <c r="C52" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D52" s="8" t="s">
+        <v>65</v>
+      </c>
+      <c r="E52" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F52" s="13"/>
+      <c r="G52" s="13"/>
+      <c r="H52" s="2"/>
+    </row>
+    <row r="53" spans="2:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="B53" s="4">
+        <v>49</v>
+      </c>
+      <c r="C53" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D53" s="8" t="s">
+        <v>66</v>
+      </c>
+      <c r="E53" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F53" s="13"/>
+      <c r="G53" s="13"/>
+      <c r="H53" s="2"/>
+    </row>
+    <row r="54" spans="2:8" ht="45" x14ac:dyDescent="0.25">
+      <c r="B54" s="4">
+        <v>50</v>
+      </c>
+      <c r="C54" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D54" s="8" t="s">
+        <v>67</v>
+      </c>
+      <c r="E54" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F54" s="13"/>
+      <c r="G54" s="13"/>
+      <c r="H54" s="2"/>
+    </row>
+    <row r="55" spans="2:8" ht="75" x14ac:dyDescent="0.25">
+      <c r="B55" s="4">
+        <v>51</v>
+      </c>
+      <c r="C55" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D55" s="8" t="s">
+        <v>68</v>
+      </c>
+      <c r="E55" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F55" s="13"/>
+      <c r="G55" s="13"/>
+      <c r="H55" s="2"/>
+    </row>
+    <row r="56" spans="2:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="B56" s="4">
+        <v>52</v>
+      </c>
+      <c r="C56" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D56" s="8" t="s">
+        <v>69</v>
+      </c>
+      <c r="E56" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F56" s="13"/>
+      <c r="G56" s="13"/>
+      <c r="H56" s="2"/>
+    </row>
+    <row r="57" spans="2:8" ht="60" x14ac:dyDescent="0.25">
+      <c r="B57" s="4">
+        <v>53</v>
+      </c>
+      <c r="C57" s="34" t="s">
+        <v>51</v>
+      </c>
+      <c r="D57" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="E57" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F57" s="13"/>
+      <c r="G57" s="13"/>
+      <c r="H57" s="2"/>
+    </row>
+    <row r="58" spans="2:8" ht="30" x14ac:dyDescent="0.25">
+      <c r="B58" s="4">
+        <v>54</v>
+      </c>
+      <c r="C58" s="34" t="s">
+        <v>38</v>
+      </c>
+      <c r="D58" s="8" t="s">
+        <v>71</v>
+      </c>
+      <c r="E58" s="13" t="s">
+        <v>52</v>
+      </c>
+      <c r="F58" s="13"/>
+      <c r="G58" s="13"/>
+      <c r="H58" s="2"/>
+    </row>
+    <row r="59" spans="2:8" ht="45.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B59" s="29">
+        <v>55</v>
+      </c>
+      <c r="C59" s="35" t="s">
+        <v>38</v>
+      </c>
+      <c r="D59" s="10" t="s">
+        <v>72</v>
+      </c>
+      <c r="E59" s="14" t="s">
+        <v>52</v>
+      </c>
+      <c r="F59" s="14"/>
+      <c r="G59" s="14"/>
+      <c r="H59" s="30"/>
+    </row>
+  </sheetData>
+  <autoFilter ref="F3:G39"/>
+  <mergeCells count="4">
+    <mergeCell ref="B2:B3"/>
+    <mergeCell ref="C2:C3"/>
+    <mergeCell ref="D2:D3"/>
+    <mergeCell ref="F2:H2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="B1:G35"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -695,25 +2020,25 @@
   <sheetData>
     <row r="1" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3"/>
     <row r="2" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="20" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="21" t="s">
+      <c r="C2" s="22" t="s">
         <v>5</v>
       </c>
-      <c r="D2" s="21" t="s">
+      <c r="D2" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="E2" s="17" t="s">
+      <c r="E2" s="18" t="s">
         <v>1</v>
       </c>
-      <c r="F2" s="17"/>
-      <c r="G2" s="18"/>
+      <c r="F2" s="18"/>
+      <c r="G2" s="19"/>
     </row>
     <row r="3" spans="2:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B3" s="20"/>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
+      <c r="B3" s="21"/>
+      <c r="C3" s="23"/>
+      <c r="D3" s="23"/>
       <c r="E3" s="11" t="s">
         <v>2</v>
       </c>
@@ -721,7 +2046,7 @@
         <v>3</v>
       </c>
       <c r="G3" s="12" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="4" spans="2:7" x14ac:dyDescent="0.25">
@@ -729,14 +2054,16 @@
         <v>1</v>
       </c>
       <c r="C4" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D4" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="E4" s="13"/>
+      <c r="E4" s="13" t="s">
+        <v>2</v>
+      </c>
       <c r="F4" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>47</v>
@@ -747,17 +2074,17 @@
         <v>2</v>
       </c>
       <c r="C5" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D5" s="5" t="s">
         <v>7</v>
       </c>
       <c r="E5" s="13"/>
       <c r="F5" s="13" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="G5" s="2" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
     </row>
     <row r="6" spans="2:7" x14ac:dyDescent="0.25">
@@ -765,7 +2092,7 @@
         <v>3</v>
       </c>
       <c r="C6" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D6" s="5" t="s">
         <v>8</v>
@@ -789,7 +2116,7 @@
       <c r="E7" s="13"/>
       <c r="F7" s="13"/>
       <c r="G7" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
@@ -805,7 +2132,7 @@
       <c r="E8" s="13"/>
       <c r="F8" s="13"/>
       <c r="G8" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
@@ -813,7 +2140,7 @@
         <v>6</v>
       </c>
       <c r="C9" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>8</v>
@@ -829,17 +2156,17 @@
         <v>7</v>
       </c>
       <c r="C10" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>35</v>
       </c>
       <c r="E10" s="13"/>
       <c r="F10" s="13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G10" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="11" spans="2:7" x14ac:dyDescent="0.25">
@@ -847,17 +2174,17 @@
         <v>8</v>
       </c>
       <c r="C11" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>11</v>
       </c>
       <c r="E11" s="13"/>
       <c r="F11" s="13" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G11" s="2" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
     </row>
     <row r="12" spans="2:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -865,10 +2192,10 @@
         <v>9</v>
       </c>
       <c r="C12" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D12" s="8" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E12" s="13" t="s">
         <v>2</v>
@@ -881,23 +2208,25 @@
         <v>10</v>
       </c>
       <c r="C13" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D13" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="E13" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="F13" s="13"/>
-      <c r="G13" s="2"/>
+      <c r="E13" s="13"/>
+      <c r="F13" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="G13" s="2" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="14" spans="2:7" x14ac:dyDescent="0.25">
       <c r="B14" s="3">
         <v>11</v>
       </c>
       <c r="C14" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D14" s="5" t="s">
         <v>13</v>
@@ -913,7 +2242,7 @@
         <v>12</v>
       </c>
       <c r="C15" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D15" s="5" t="s">
         <v>14</v>
@@ -939,7 +2268,7 @@
       </c>
       <c r="F16" s="13"/>
       <c r="G16" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="17" spans="2:7" x14ac:dyDescent="0.25">
@@ -957,7 +2286,7 @@
       </c>
       <c r="F17" s="13"/>
       <c r="G17" s="2" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="18" spans="2:7" ht="45" x14ac:dyDescent="0.25">
@@ -965,7 +2294,7 @@
         <v>15</v>
       </c>
       <c r="C18" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D18" s="8" t="s">
         <v>16</v>
@@ -981,7 +2310,7 @@
         <v>16</v>
       </c>
       <c r="C19" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D19" s="8" t="s">
         <v>15</v>
@@ -997,7 +2326,7 @@
         <v>17</v>
       </c>
       <c r="C20" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D20" s="5" t="s">
         <v>17</v>
@@ -1013,7 +2342,7 @@
         <v>18</v>
       </c>
       <c r="C21" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D21" s="5" t="s">
         <v>18</v>
@@ -1029,7 +2358,7 @@
         <v>19</v>
       </c>
       <c r="C22" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D22" s="5" t="s">
         <v>19</v>
@@ -1045,7 +2374,7 @@
         <v>20</v>
       </c>
       <c r="C23" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D23" s="8" t="s">
         <v>20</v>
@@ -1061,7 +2390,7 @@
         <v>21</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D24" s="5" t="s">
         <v>21</v>
@@ -1077,7 +2406,7 @@
         <v>22</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D25" s="9" t="s">
         <v>22</v>
@@ -1093,7 +2422,7 @@
         <v>23</v>
       </c>
       <c r="C26" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D26" s="5" t="s">
         <v>23</v>
@@ -1109,7 +2438,7 @@
         <v>24</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D27" s="8" t="s">
         <v>24</v>
@@ -1119,7 +2448,7 @@
       </c>
       <c r="F27" s="13"/>
       <c r="G27" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
     </row>
     <row r="28" spans="2:7" ht="31.5" customHeight="1" x14ac:dyDescent="0.25">
@@ -1137,7 +2466,7 @@
       </c>
       <c r="F28" s="13"/>
       <c r="G28" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="29" spans="2:7" x14ac:dyDescent="0.25">
@@ -1155,7 +2484,7 @@
       </c>
       <c r="F29" s="13"/>
       <c r="G29" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="30" spans="2:7" ht="45" x14ac:dyDescent="0.25">
@@ -1173,7 +2502,7 @@
       </c>
       <c r="F30" s="13"/>
       <c r="G30" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="31" spans="2:7" x14ac:dyDescent="0.25">
@@ -1191,7 +2520,7 @@
       </c>
       <c r="F31" s="13"/>
       <c r="G31" s="2" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="32" spans="2:7" ht="45" x14ac:dyDescent="0.25">
@@ -1204,18 +2533,20 @@
       <c r="D32" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="E32" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="F32" s="13"/>
-      <c r="G32" s="2"/>
+      <c r="E32" s="13"/>
+      <c r="F32" s="13" t="s">
+        <v>43</v>
+      </c>
+      <c r="G32" s="2" t="s">
+        <v>44</v>
+      </c>
     </row>
     <row r="33" spans="2:7" ht="30" x14ac:dyDescent="0.25">
       <c r="B33" s="3">
         <v>30</v>
       </c>
       <c r="C33" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D33" s="8" t="s">
         <v>32</v>
@@ -1225,7 +2556,7 @@
       </c>
       <c r="F33" s="13"/>
       <c r="G33" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="34" spans="2:7" ht="30" x14ac:dyDescent="0.25">
@@ -1233,7 +2564,7 @@
         <v>31</v>
       </c>
       <c r="C34" s="5" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D34" s="8" t="s">
         <v>33</v>
@@ -1243,7 +2574,7 @@
       </c>
       <c r="F34" s="13"/>
       <c r="G34" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="35" spans="2:7" ht="30.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -1251,16 +2582,18 @@
         <v>32</v>
       </c>
       <c r="C35" s="7" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D35" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="E35" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="F35" s="14"/>
-      <c r="G35" s="16"/>
+      <c r="E35" s="14"/>
+      <c r="F35" s="14" t="s">
+        <v>43</v>
+      </c>
+      <c r="G35" s="16" t="s">
+        <v>44</v>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="E3:F35"/>

</xml_diff>